<commit_message>
Selejtkezelés rendbetétele és megjelenítés tisztázása
</commit_message>
<xml_diff>
--- a/adatok/termekadatok.xlsx
+++ b/adatok/termekadatok.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\csadr\Desktop\koltseg_kalkulator\adatok\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{349476FB-28B2-4D31-A0CE-42FB6D279105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09AAC62D-7EBC-4822-8011-E83591F69426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{4F13D512-5F0F-4C51-8B85-569053DA9FC2}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="15345" xr2:uid="{4F13D512-5F0F-4C51-8B85-569053DA9FC2}"/>
   </bookViews>
   <sheets>
     <sheet name="Adatok" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>eladasi_ar</t>
   </si>
@@ -101,9 +101,6 @@
   </si>
   <si>
     <t>PLA</t>
-  </si>
-  <si>
-    <t>nem</t>
   </si>
   <si>
     <t>W (becsült átlagos fogyasztás)</t>
@@ -577,14 +574,17 @@
       <c r="H2" s="5">
         <v>5000</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>22</v>
+      <c r="I2" s="5">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I890" xr:uid="{E150FA40-E346-4174-9697-E3458B4573DB}">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I890" xr:uid="{E150FA40-E346-4174-9697-E3458B4573DB}">
       <formula1>"igen,nem"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{B50D28DA-7C2E-4AF1-AF93-A67AAC720DA4}">
+      <formula1>"0,1,2,3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -620,7 +620,7 @@
         <v>61.33</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -631,7 +631,7 @@
         <v>150</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -660,12 +660,12 @@
         <v>10</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B7" s="2">
         <v>27</v>
@@ -676,7 +676,7 @@
     </row>
     <row r="8" spans="1:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B8" s="2">
         <v>120</v>

</xml_diff>

<commit_message>
Koltsegkalkulator javitasa es dokumentacio frissitese
</commit_message>
<xml_diff>
--- a/adatok/termekadatok.xlsx
+++ b/adatok/termekadatok.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\csadr\Desktop\koltseg_kalkulator\adatok\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC13802-CD3A-40A1-85CF-106FE3BA9B7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{595A829C-8FC3-4270-80B3-968B6B013025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4F13D512-5F0F-4C51-8B85-569053DA9FC2}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{4F13D512-5F0F-4C51-8B85-569053DA9FC2}"/>
   </bookViews>
   <sheets>
     <sheet name="Adatok" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>eladasi_ar</t>
   </si>
@@ -82,13 +82,7 @@
     <t>platform_jutalek</t>
   </si>
   <si>
-    <t>Ft/hó</t>
-  </si>
-  <si>
     <t>Ft</t>
-  </si>
-  <si>
-    <t>havi_fix_koltseg</t>
   </si>
   <si>
     <t>indulo_beruhazas</t>
@@ -212,9 +206,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-téma">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022 téma">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -252,7 +246,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -358,7 +352,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -500,7 +494,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -548,7 +542,7 @@
         <v>0</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
@@ -556,10 +550,10 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C2" s="5">
         <v>7000</v>
@@ -599,7 +593,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BA079A-B265-4007-8B45-2ACA07F84F2B}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
@@ -623,10 +617,10 @@
         <v>12</v>
       </c>
       <c r="B2" s="2">
-        <v>61.33</v>
+        <v>61.327399999999997</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -637,53 +631,46 @@
         <v>150</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="2"/>
+        <v>16</v>
+      </c>
+      <c r="B4" s="2">
+        <v>90943</v>
+      </c>
       <c r="C4" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="2"/>
+        <v>14</v>
+      </c>
+      <c r="B5" s="2">
+        <v>11.07</v>
+      </c>
       <c r="C5" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B6" s="2">
-        <v>11.07</v>
+        <v>4.43</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="2">
-        <v>4.43</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
+    <row r="7" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>